<commit_message>
결과 파일 업데이트 2026-09-01 06:24
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260901.xlsx
+++ b/results/andar_할인율모니터링_20260901.xlsx
@@ -937,7 +937,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10,032</t>
+          <t>10,033</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3,509</t>
+          <t>3,510</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3,509</t>
+          <t>3,510</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>233</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1117,153 +1117,153 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9620&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17443&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EMTBG-12</t>
+          <t>EPTSC-04</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>데일리 쇼퍼백</t>
+          <t>[3 SET] 필라테스 삭스</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>41,700</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>30,900</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1,395</t>
+          <t>367</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13838&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17443&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EOTFB-01</t>
+          <t>EPTSC-05</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>에어쿨링 서스테이너블 와이드 헤드밴드</t>
+          <t>[3 SET] 필라테스 삭스</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>41,700</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>30,900</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2,343</t>
+          <t>367</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14076&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17443&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EOTBG-13</t>
+          <t>EPTSC-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>멀티 포켓 숄더 앤 크로스백</t>
+          <t>[3 SET] 필라테스 삭스</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>63,000</t>
+          <t>41,700</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>63,000</t>
+          <t>30,900</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>367</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10478&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9620&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ENTBG-05</t>
+          <t>EMTBG-12</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>미니 숄더 앤 크로스백</t>
+          <t>데일리 쇼퍼백</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1273,39 +1273,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5,100</t>
+          <t>1,396</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13838&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ENTBG-03</t>
+          <t>EOTFB-01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>데일리 스트링 쇼퍼백</t>
+          <t>에어쿨링 서스테이너블 와이드 헤드밴드</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1315,39 +1315,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>719</t>
+          <t>2,343</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17414&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14076&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EPTBG-01</t>
+          <t>EOTBG-13</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>에어플라이 프리런 러닝 벨트</t>
+          <t>멀티 포켓 숄더 앤 크로스백</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>63,000</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>63,000</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1357,39 +1357,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>409</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EOTBG-21</t>
+          <t>ENTBG-03</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>데일리 라운드백</t>
+          <t>데일리 스트링 쇼퍼백</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1399,39 +1399,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>719</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16868&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10478&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EPTBG-03</t>
+          <t>ENTBG-05</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>컴팩트 포켓 크로스백</t>
+          <t>미니 숄더 앤 크로스백</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1441,133 +1441,133 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>5,101</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17443&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17414&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EPTSC-04</t>
+          <t>EPTBG-01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[3 SET] 필라테스 삭스</t>
+          <t>에어플라이 프리런 러닝 벨트</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>41,700</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>30,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>55</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17443&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EPTSC-05</t>
+          <t>EOTBG-21</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[3 SET] 필라테스 삭스</t>
+          <t>데일리 라운드백</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>41,700</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>30,900</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>103</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17443&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EPTSC-06</t>
+          <t>EJFST-02</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>[3 SET] 필라테스 삭스</t>
+          <t>릴렉스 요가링</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>41,700</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>30,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>367</t>
+          <t>6,565</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1579,27 +1579,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16868&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EJFST-02</t>
+          <t>EPTBG-03</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>릴렉스 요가링</t>
+          <t>컴팩트 포켓 크로스백</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1609,96 +1609,96 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>6,565</t>
+          <t>116</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15372&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8817&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EOTBG-16</t>
+          <t>EMTSC-03</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>폴더블 미니백 2.0</t>
+          <t>[1&amp;1] 논슬립 서포트 풀 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>17,800</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>4,812</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8817&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15372&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EMTSC-03</t>
+          <t>EOTBG-16</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 풀 토삭스 (HOLE)</t>
+          <t>폴더블 미니백 2.0</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>17,800</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>4,812</t>
+          <t>281</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -1747,27 +1747,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13862&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EOTBG-03</t>
+          <t>EPTCP-03</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>데이 앤 트래블 숄더백</t>
+          <t>썬가드 와이드 버킷햇</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1777,123 +1777,123 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>57</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8838&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13862&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EMTSV-03</t>
+          <t>EOTBG-03</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 무릎 보호대</t>
+          <t>데이 앤 트래블 숄더백</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>22,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1,986</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13852&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8838&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>EMTSV-03</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>라이트 러닝 베스트</t>
+          <t>[1&amp;1] 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>22,900</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>1,986</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EPTCP-03</t>
+          <t>EOTBG-10</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>썬가드 와이드 버킷햇</t>
+          <t>에어플라이 투웨이 프리런 백 3.0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1903,39 +1903,39 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>1,130</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13852&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EOTBG-10</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>에어플라이 투웨이 프리런 백 3.0</t>
+          <t>라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>1,129</t>
+          <t>98</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -2125,27 +2125,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14563&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16629&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EOTMK-01</t>
+          <t>EPTET-01</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>UV 프로텍션 골프 마스크 (벨크로)</t>
+          <t>언더웨어 파우치</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2155,12 +2155,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>1,097</t>
+          <t>328</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>693</t>
+          <t>694</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2209,27 +2209,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16629&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14563&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EPTET-01</t>
+          <t>EOTMK-01</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>언더웨어 파우치</t>
+          <t>UV 프로텍션 골프 마스크 (벨크로)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2239,12 +2239,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>1,097</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -2335,79 +2335,79 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EMTET-02</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>소프트 쿠셔닝 훌라후프</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>15,800</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>616</t>
+          <t>3,177</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15369&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EOTBG-19</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>위켄드 호보백</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>15,800</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>3,177</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2419,79 +2419,79 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EMTET-02</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>소프트 쿠셔닝 훌라후프</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>15,800</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>3,177</t>
+          <t>617</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15369&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>EOTBG-19</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>위켄드 호보백</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>15,800</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>3,177</t>
+          <t>61</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2545,27 +2545,27 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15370&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8726&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EOTBG-14</t>
+          <t>EMTSC-03</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>폴더블 캐리백 2.0</t>
+          <t>논슬립 서포트 풀 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2575,39 +2575,39 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>4,812</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8726&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EMTSC-03</t>
+          <t>EOTSC-15</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>논슬립 서포트 풀 토삭스 (HOLE)</t>
+          <t>논슬립 퍼포먼스 풀 토삭스</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2617,39 +2617,39 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>4,812</t>
+          <t>149</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EOTSC-15</t>
+          <t>EPTSC-06</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 풀 토삭스</t>
+          <t>필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2659,39 +2659,39 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15370&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EKPMT-03</t>
+          <t>EOTBG-14</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>릴렉스 논슬립 요가 타월</t>
+          <t>폴더블 캐리백 2.0</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>35,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>35,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2701,39 +2701,39 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>1,545</t>
+          <t>86</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EOTBG-12</t>
+          <t>EPTSV-03</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>프리런 벨크로 러닝 벨트</t>
+          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2743,39 +2743,39 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>234</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EPTSC-06</t>
+          <t>EOTBG-17</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>필라테스 크루 삭스</t>
+          <t>3 in 1 캐리온 더플백</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>109,000</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>109,000</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2785,39 +2785,39 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>39</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EOTBG-17</t>
+          <t>EKPMT-03</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>3 in 1 캐리온 더플백</t>
+          <t>릴렉스 논슬립 요가 타월</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>109,000</t>
+          <t>35,900</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>109,000</t>
+          <t>35,900</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2827,39 +2827,39 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>1,545</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EPTSV-03</t>
+          <t>EOTBG-12</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
+          <t>프리런 벨크로 러닝 벨트</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2869,19 +2869,19 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>243</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2891,32 +2891,32 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>컴프레션 러닝 니삭스</t>
+          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>662</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2975,59 +2975,59 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
+          <t>컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>662</t>
+          <t>341</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EPTFB-02</t>
+          <t>EOTBG-23</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>퍼포먼스 심리스 손목밴드</t>
+          <t>안다르 실버 리유저블백 M</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3037,39 +3037,39 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>262</t>
+          <t>359</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EOTBG-23</t>
+          <t>EPTFB-02</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>안다르 실버 리유저블백 M</t>
+          <t>퍼포먼스 심리스 손목밴드</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3079,12 +3079,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>359</t>
+          <t>262</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -3133,27 +3133,27 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EOTSV-03</t>
+          <t>ENTSC-20</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>서포트 허리 보호대</t>
+          <t>시그니처 로고 크루 삭스</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3163,39 +3163,39 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>562</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ENTSC-20</t>
+          <t>EPTSC-04</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>시그니처 로고 크루 삭스</t>
+          <t>필라테스 토삭스</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>93</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -3259,27 +3259,27 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EOTGL-01</t>
+          <t>EOTSV-03</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>짐 글러브 2.0</t>
+          <t>서포트 허리 보호대</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3289,39 +3289,39 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>172</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EPTSC-04</t>
+          <t>EOTGL-01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>필라테스 토삭스</t>
+          <t>짐 글러브 2.0</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>284</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3343,27 +3343,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EKPMB-01</t>
+          <t>EMTRB-01</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>릴렉스 웨이트볼 0.5kg</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3373,12 +3373,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>687</t>
+          <t>1,364</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3390,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EMTRB-01</t>
+          <t>EMTRB-02</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EMTRB-02</t>
+          <t>EMTRB-03</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3469,27 +3469,27 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EMTRB-03</t>
+          <t>EKPMB-01</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>릴렉스 웨이트볼 0.5kg</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3499,12 +3499,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>1,364</t>
+          <t>687</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3709,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>184</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>706</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>1,320</t>
+          <t>1,321</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4015,79 +4015,79 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EKPMB-02</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>릴렉스 미니 짐볼</t>
+          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>17,800</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>1,222</t>
+          <t>3,017</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 크루삭스</t>
+          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>17,800</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>662</t>
+          <t>3,017</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4099,79 +4099,79 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>EKPMB-02</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
+          <t>릴렉스 미니 짐볼</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>17,800</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>3,017</t>
+          <t>1,222</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
+          <t>논슬립 퍼포먼스 크루삭스</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>17,800</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>3,017</t>
+          <t>662</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>747</t>
+          <t>748</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4225,27 +4225,27 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12765&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>ENTBG-16</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
+          <t>라이트 패딩 쇼퍼백</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>620</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4267,27 +4267,27 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12765&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16640&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ENTBG-16</t>
+          <t>EPTBG-05</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>라이트 패딩 쇼퍼백</t>
+          <t>안다르 시그니처 로고 에코백</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4297,39 +4297,39 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EPTSC-02</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>하이 쿠션 테이핑 러닝 삭스</t>
+          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4339,39 +4339,39 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>557</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ENTMK-01</t>
+          <t>EKPRB-04</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>UV 프로텍션 맨즈 골프 마스크</t>
+          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4381,39 +4381,39 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>1,531</t>
+          <t>467</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EMTSC-27</t>
+          <t>ENTMK-01</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>올라운드 오버 니삭스</t>
+          <t>UV 프로텍션 맨즈 골프 마스크</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4423,39 +4423,39 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>1,531</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EKPRB-04</t>
+          <t>EPTSC-02</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
+          <t>하이 쿠션 테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>467</t>
+          <t>87</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4477,79 +4477,79 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EMTSC-27</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
+          <t>올라운드 오버 니삭스</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>41,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>35,600</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>592</t>
+          <t>292</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>EOTSC-01</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>프레시 필드 니삭스</t>
+          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>41,800</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>35,600</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>294</t>
+          <t>593</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4561,27 +4561,27 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>ENTSC-12</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>맨즈 라이트 러닝 베스트</t>
+          <t>논슬립 퍼포먼스 토삭스</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4591,39 +4591,39 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4,134</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ENTSC-12</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 토삭스</t>
+          <t>맨즈 라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4633,12 +4633,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>4,134</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4675,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>693</t>
+          <t>694</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4687,27 +4687,27 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EMTSV-03</t>
+          <t>EPTET-03</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>서포트 무릎 보호대</t>
+          <t>안다르 3단 양우산</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4717,12 +4717,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>1,986</t>
+          <t>35</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.4</t>
         </is>
       </c>
     </row>
@@ -4771,27 +4771,27 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>논슬립 스킨 하프 토삭스</t>
+          <t>서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4801,91 +4801,91 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>706</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EPTET-03</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>안다르 3단 양우산</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>301</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>서포트 발목 보호대</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>301</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -4897,247 +4897,247 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EMTSV-03</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>1,986</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>논슬립 스킨 하프 토삭스</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>105</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
+          <t>[1&amp;1] 3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>25,900</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>545</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 팔토시</t>
+          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>25,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>545</t>
+          <t>643</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ENTSC-07</t>
+          <t>EOTSC-10</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>[3 SET] 에어컴피 크루 삭스</t>
+          <t>시그니처 로고 맨즈 크루 삭스</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>51,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>212</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17522&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>ENTSC-07</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 필라테스 삭스</t>
+          <t>[3 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>51,000</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>556</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>EPTSC-08</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5191,59 +5191,59 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17522&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>EPTSC-08</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 니삭스</t>
+          <t>[1&amp;1] 맨즈 필라테스 삭스</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>752</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>EPTSC-05</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>필라테스 앵클 삭스</t>
+          <t>논슬립 퍼포먼스 니삭스</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -5263,91 +5263,91 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>752</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>EPTSC-05</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
+          <t>필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>35</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EOTSC-10</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>시그니처 로고 맨즈 크루 삭스</t>
+          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>154</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -5359,79 +5359,79 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10657&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EOTGL-02</t>
+          <t>EMTSC-17</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>히트 런 글러브</t>
+          <t>[3 SET] 맨즈 클래식 삭스</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>20,700</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>223</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EOTGL-02</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
+          <t>히트 런 글러브</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>22,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>212</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -5443,42 +5443,42 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10657&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EMTSC-17</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>[3 SET] 맨즈 클래식 삭스</t>
+          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>20,700</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>22,900</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>588</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -5737,69 +5737,69 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9612&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>EOTET-01</t>
+          <t>EMTSC-28</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>소프트 뱀부 롱 타월</t>
+          <t>[1&amp;1] 리브드 셔링 루즈 삭스</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>395</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16640&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EPTBG-05</t>
+          <t>EOTET-01</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>안다르 시그니처 로고 에코백</t>
+          <t>소프트 뱀부 롱 타월</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -5809,12 +5809,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>236</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5863,69 +5863,69 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9612&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EMTSC-28</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>[1&amp;1] 리브드 셔링 루즈 삭스</t>
+          <t>릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>395</t>
+          <t>593</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 1kg</t>
+          <t>논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -5935,39 +5935,39 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>593</t>
+          <t>85</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>EOTSC-01</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>논슬립 스킨 토삭스</t>
+          <t>프레시 필드 니삭스</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -5977,12 +5977,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>294</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -6157,79 +6157,79 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>[1&amp;1] 레그 워머</t>
+          <t>서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>588</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16036&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>EOTCP-06</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>[1&amp;1] 레그 워머</t>
+          <t>소프트 니트 버킷햇</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>52</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -6241,37 +6241,37 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16036&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>EOTCP-06</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>소프트 니트 버킷햇</t>
+          <t>[1&amp;1] 레그 워머</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>230</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -6283,42 +6283,42 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>서포트 팔꿈치 보호대</t>
+          <t>[1&amp;1] 레그 워머</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>230</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -6451,27 +6451,27 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17436&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EPTSV-01</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>램스울 크루 삭스</t>
+          <t>3D 쿨링 핑거홀 팔토시</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -6481,39 +6481,39 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>178</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14562&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EOTBG-11</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>메쉬 파우치</t>
+          <t>램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -6523,29 +6523,29 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>315</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12480&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14562&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>ENTSC-24</t>
+          <t>EOTBG-11</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>웜 슬릿 레그 워머</t>
+          <t>메쉬 파우치</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -6565,39 +6565,39 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>190</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12480&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>ENTMU-01</t>
+          <t>ENTSC-24</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>소프트 니트 머플러</t>
+          <t>웜 슬릿 레그 워머</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6607,81 +6607,81 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>472</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10939&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>EMTSC-29</t>
+          <t>ENTSC-07</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>니트 루즈 삭스</t>
+          <t>에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>17,000</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>513</t>
+          <t>556</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12783&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>ENTSC-26</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>니트 기모 오버 니삭스</t>
+          <t>데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -6703,69 +6703,69 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17436&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EPTSV-01</t>
+          <t>EOTSC-18</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>3D 쿨링 핑거홀 팔토시</t>
+          <t>[1&amp;1] 올데이 기모 삭스</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
+          <t>21,800</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
           <t>15,900</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>15,900</t>
-        </is>
-      </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>225</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15734&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>ENTMU-01</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>레그 미들 워머</t>
+          <t>소프트 니트 머플러</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6775,81 +6775,81 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>472</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10939&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ENTSC-07</t>
+          <t>EMTSC-29</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>에어컴피 크루 삭스</t>
+          <t>니트 루즈 삭스</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>17,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>513</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12783&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>ENTSC-26</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>데일리 루즈 삭스</t>
+          <t>니트 기모 오버 니삭스</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6859,7 +6859,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>354</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -6871,27 +6871,27 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15734&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>EOTMU-01</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>스트링 패딩 넥워머</t>
+          <t>레그 미들 워머</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -6901,39 +6901,39 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16035&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>EOTSC-12</t>
+          <t>EOTMU-01</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>소프트 니트 기모 니삭스</t>
+          <t>스트링 패딩 넥워머</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6943,39 +6943,39 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>46</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16034&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16035&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>EOTGL-03</t>
+          <t>EOTSC-12</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>소프트 니트 플립 글러브</t>
+          <t>소프트 니트 기모 니삭스</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -6985,54 +6985,54 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>101</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16034&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>EOTSC-18</t>
+          <t>EOTGL-03</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>[1&amp;1] 올데이 기모 삭스</t>
+          <t>소프트 니트 플립 글러브</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>83</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -7081,27 +7081,27 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15733&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>EOTSC-11</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>웜 레그 롱 워머</t>
+          <t>레그 숏 워머</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -7123,27 +7123,27 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15733&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EOTSC-11</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>레그 숏 워머</t>
+          <t>웜 레그 롱 워머</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">

</xml_diff>